<commit_message>
chore: Modificação de importação de arquivos
</commit_message>
<xml_diff>
--- a/frontend/public/modelo_importacao_ativos.xlsx
+++ b/frontend/public/modelo_importacao_ativos.xlsx
@@ -8,9 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ATIVOS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POOLS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CATEGORIAS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUÇÕES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ATIVOS'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ATIVOS'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,8 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +36,15 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <color rgb="000000FF"/>
+    </font>
+    <font>
+      <color rgb="00008000"/>
+    </font>
+    <font>
+      <color rgb="00666666"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -41,7 +55,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
+        <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,11 +71,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,63 +449,510 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" style="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>patrimonio</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pool</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>categoria</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>fabricante</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>modelo</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>preco</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>localizacao</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TI-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Notebook corporativo</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Equipamento de uso interno</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Dell</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Latitude 5450</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>6500</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Matriz</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>João da Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TI-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Monitor 24 polegadas</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Monitor para estação de trabalho</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>LG</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>24MP400</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>899.9</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Matriz</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Maria Souza</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ADM-0001</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Cadeira ergonômica</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Administrativo</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Cadeira para escritório</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Flexform</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Uni</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1450</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Matriz</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Lima</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>POOLS DISPONÍVEIS - EXEMPLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>RH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Administrativo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>CATEGORIAS DISPONÍVEIS - EXEMPLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Desktop</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Impressora</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Servidor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Roteador</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Access Point</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Nobreak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Celular</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Projetor</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Telefone</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Mobiliário</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Ar-condicionado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Veículo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Ferramenta</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>INSTRUÇÃO</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>DETALHE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>1. Preencha ATIVOS</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Patrimônio, nome, pool e categoria são obrigatórios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>2. Pool e Categoria</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Devem existir no sistema. Erros de digitação são rejeitados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>3. Validação</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Use a tela Importações &gt; Analisar arquivo antes de gravar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>4. Linhas inválidas</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Não são cadastradas. O sistema mostra o motivo da rejeição.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>5. Modelo atualizado</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Prefira baixar o modelo pela própria tela do sistema; ele contém os Pools e Categorias atuais.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>